<commit_message>
Add agg_plan_month_provider_type_claim_volume spec to agg_curation
Include the exploration queries that check which provider types appear in claims and whether any claim has lines from more than one provider type.
</commit_message>
<xml_diff>
--- a/docs/agg_curation.xlsx
+++ b/docs/agg_curation.xlsx
@@ -4,11 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12240"/>
+    <workbookView windowWidth="28800" windowHeight="12240" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="agg_plan_month_cost" sheetId="1" r:id="rId1"/>
-    <sheet name="singular_tests" sheetId="2" r:id="rId2"/>
+    <sheet name="agg_plan_month_claim_volume" sheetId="3" r:id="rId2"/>
+    <sheet name="singular_tests" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="176">
   <si>
     <t>agg_plan_month_cost | Model Curation Specification</t>
   </si>
@@ -279,10 +280,158 @@
     <t>Paid amounts: DECIMAL(38,2). member_month_count: INTEGER (cast in final). fractional_member_months and all four PMPM ratios: DOUBLE. Grain and plan attributes: VARCHAR and DATE.</t>
   </si>
   <si>
-    <t>agg_plan_month_cost | Singular Test Specifications</t>
-  </si>
-  <si>
-    <t>Scope: Five singular tests for model grain, claim amounts, enrollment measures, and PMPM formulas</t>
+    <t>agg_plan_month_provider_type_claim_volume | Model Curation Specification</t>
+  </si>
+  <si>
+    <t>Grain: One row per plan_id + month_start_date (service month) + billing_provider_type (i.e., HOSP, LAB, PHYS, SNF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scope: Include paid, eligibility-matched claims with service dates on or before the analysis cutoff. Aggregate claim volume by service month and billing provider type. Include all four provider types for each enrolled plan-month, even when there are no qualifying claims.
+</t>
+  </si>
+  <si>
+    <t>Plan-month-provider-type keys from enrolled plan-months × provider types, union qualifying claim keys</t>
+  </si>
+  <si>
+    <t>Claim plan_id attributed using service-date eligibility; unmatched paid claims excluded</t>
+  </si>
+  <si>
+    <t>Enrollment month or service_from_month_start_date</t>
+  </si>
+  <si>
+    <t>First day of service reporting month; no payment-month claim-volume view</t>
+  </si>
+  <si>
+    <t>billing_provider_type</t>
+  </si>
+  <si>
+    <t>fct_medical_claim_lines; defined domain</t>
+  </si>
+  <si>
+    <t>HOSP, LAB, PHYS, SNF</t>
+  </si>
+  <si>
+    <t>Include all four types for every enrolled plan-month, even when claim counts are zero</t>
+  </si>
+  <si>
+    <t>claim_line_count</t>
+  </si>
+  <si>
+    <t>count(*) by service-date plan_id, service_from_month_start_date, billing_provider_type</t>
+  </si>
+  <si>
+    <t>Zero when no qualifying paid claim lines; additive across provider types</t>
+  </si>
+  <si>
+    <t>claim_count</t>
+  </si>
+  <si>
+    <t>count(distinct claim_id) by service-date plan_id, service_from_month_start_date, billing_provider_type</t>
+  </si>
+  <si>
+    <t>Zero when no qualifying claims. In current data, no qualifying claim spans provider types; check plan and month attribution before treating claim_count as fully additive</t>
+  </si>
+  <si>
+    <t>count(*) by plan_id and month_start_date; repeat on each provider-type row</t>
+  </si>
+  <si>
+    <t>Plan-month denominator repeated across provider types; do not sum across provider types</t>
+  </si>
+  <si>
+    <t>sum(member_month_exposure) by plan_id and month_start_date; repeat on each provider-type row</t>
+  </si>
+  <si>
+    <t>Prorated exposure, unrounded; repeated across provider types; do not sum across provider types</t>
+  </si>
+  <si>
+    <t>claim_lines_per_1000_member_months</t>
+  </si>
+  <si>
+    <t>claim_line_count * 1000.0 / nullif(member_month_count, 0)</t>
+  </si>
+  <si>
+    <t>Null without enrollment; non-additive rate; recalculate on rollup</t>
+  </si>
+  <si>
+    <t>claims_per_1000_member_months</t>
+  </si>
+  <si>
+    <t>claim_count * 1000.0 / nullif(member_month_count, 0)</t>
+  </si>
+  <si>
+    <t>Include every enrolled plan-month × each of HOSP, LAB, PHYS, SNF, even without claims. Defensively include qualifying claim plan-month-provider-type combinations not represented by enrollment; investigate any such exceptions. Do not generate payment-only months.</t>
+  </si>
+  <si>
+    <t>Qualifying claims</t>
+  </si>
+  <si>
+    <t>Filter claim_status_code = 'PAID', has_matching_eligibility, and service_from_date &lt;= analysis_through_date; use the service-date plan_id. Current qualifying population: 39,231 claim lines.</t>
+  </si>
+  <si>
+    <t>Provider-type domain</t>
+  </si>
+  <si>
+    <t>HOSP, LAB, PHYS, SNF all occur in qualifying claims. Generate zero-claim rows from a fixed list of these four types in the model; the list matches the accepted_values test on billing_provider_type in _stg_models.yml.</t>
+  </si>
+  <si>
+    <t>Use service_from_month_start_date exclusively; payment month is not used for claim counts or rates.</t>
+  </si>
+  <si>
+    <t>Claim-count caveat</t>
+  </si>
+  <si>
+    <t>Current qualifying data has no claim_id with more than one billing_provider_type. Verify whether claim_id can span plan_id or service month before describing claim_count as additive across all dimensions.</t>
+  </si>
+  <si>
+    <t>Coalesce missing claim_line_count, claim_count, member_month_count, and fractional_member_months to zero; use nullif(member_month_count, 0) for rates. Zero-claim enrolled rows have zero rates. Defensive claim-only rows without enrollment have null rates and should be investigated.</t>
+  </si>
+  <si>
+    <t>Repeated denominators</t>
+  </si>
+  <si>
+    <t>member_month_count and fractional_member_months repeat on each provider-type row of the same plan-month. Never sum them across provider types; use one plan-month denominator when rolling up provider types.</t>
+  </si>
+  <si>
+    <t>Claim-volume reconciliation</t>
+  </si>
+  <si>
+    <t>Reconcile claim_line_count and claim_count to the qualifying claim-line fact by plan_id, service month, and provider type; check missing and extra keys, including zero-claim rows.</t>
+  </si>
+  <si>
+    <t>Enrollment reconciliation</t>
+  </si>
+  <si>
+    <t>For each plan-month-provider-type row, compare both denominators to agg_plan_month_cost at the same plan-month; verify identical denominators across provider types.</t>
+  </si>
+  <si>
+    <t>Sum claim lines and appropriate distinct-claim counts at the desired rollup grain; use unduplicated plan-month denominators and recalculate rates. Never sum or average rates.</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>Exclude units because units are not consistently comparable across HOSP, LAB, PHYS, and SNF. Claim lines are a volume proxy, not necessarily encounters or services.</t>
+  </si>
+  <si>
+    <t>analysis_through_date = 2026-06-30; no payment-month extension in claim-volume reporting.</t>
+  </si>
+  <si>
+    <t>Five singular tests documented in the singular_tests tab: unique grain, claim-count reconciliation, enrollment reconciliation to agg_plan_month_cost, provider-type completeness, and rate formulas. Add generic not_null and plan relationships tests.</t>
+  </si>
+  <si>
+    <t>Claim counts and member_month_count: INTEGER; fractional_member_months and claim-volume rates: DOUBLE; grain and plan attributes: VARCHAR and DATE. Confirm implemented casts.</t>
+  </si>
+  <si>
+    <t>Metric scope</t>
+  </si>
+  <si>
+    <t>Core rates use member_month_count as denominator. Fractional-denominator rates are deferred unless reporting requirements justify them.</t>
+  </si>
+  <si>
+    <t>Aggregate models | Singular Test Specifications</t>
+  </si>
+  <si>
+    <t>Scope: Ten singular tests for agg_plan_month_cost and agg_plan_month_provider_type_claim_volume: grain, reconciliations, row completeness, and ratio formulas</t>
   </si>
   <si>
     <t>Test name</t>
@@ -352,6 +501,63 @@
   </si>
   <si>
     <t>Tolerance 1e-6; covers both service/payment bases and count/fractional denominators.</t>
+  </si>
+  <si>
+    <t>assert_agg_plan_month_provider_type_claim_volume_unique_grain</t>
+  </si>
+  <si>
+    <t>agg_plan_month_provider_type_claim_volume</t>
+  </si>
+  <si>
+    <t>No duplicate (plan_id, month_start_date, billing_provider_type) combinations</t>
+  </si>
+  <si>
+    <t>Complement generic not_null tests for all three grain columns.</t>
+  </si>
+  <si>
+    <t>assert_agg_plan_month_provider_type_claim_volume_claim_counts_reconcile_to_claims</t>
+  </si>
+  <si>
+    <t>agg_plan_month_provider_type_claim_volume; fct_medical_claim_lines</t>
+  </si>
+  <si>
+    <t>Compare claim_line_count = count(*) and claim_count = count(distinct claim_id) with qualifying claim lines (PAID, eligibility-matched, service_from_date &lt;= analysis_through_date), aggregated by service-date plan_id, service_from_month_start_date, and billing_provider_type; use full outer comparison, and flag null counts. Treat a missing source key as zero so zero-claim rows are not flagged.</t>
+  </si>
+  <si>
+    <t>Integer counts; exact comparison. Detects missing, extra, and mismatched plan-month-provider-type rows.</t>
+  </si>
+  <si>
+    <t>assert_agg_plan_month_provider_type_claim_volume_enrollment_reconciles_to_agg_plan_month_cost</t>
+  </si>
+  <si>
+    <t>agg_plan_month_provider_type_claim_volume; agg_plan_month_cost</t>
+  </si>
+  <si>
+    <t>For every row, compare member_month_count and fractional_member_months with agg_plan_month_cost at the same plan_id and month_start_date; flag null measures. Claim-only rows without enrollment must show zero.</t>
+  </si>
+  <si>
+    <t>Comparing each provider-type row to one plan-month value also verifies the denominators are identical across provider types; tolerance 1e-9 for fractional exposure.</t>
+  </si>
+  <si>
+    <t>assert_agg_plan_month_provider_type_claim_volume_provider_types_complete</t>
+  </si>
+  <si>
+    <t>agg_plan_month_provider_type_claim_volume; fct_member_plan_month</t>
+  </si>
+  <si>
+    <t>For every distinct enrolled (plan_id, month_start_date) in fct_member_plan_month, verify that the claim-volume aggregate contains exactly four rows: one each for HOSP, LAB, PHYS, and SNF. Detect enrolled plan-months missing entirely from the aggregate as well as missing or duplicate provider types.</t>
+  </si>
+  <si>
+    <t>Use source enrollment plan-months as the starting population, not just plan-months already present in the claim-volume aggregate. Enforces zero-claim rows for all four provider types.</t>
+  </si>
+  <si>
+    <t>assert_agg_plan_month_provider_type_claim_volume_rates_match_formulas</t>
+  </si>
+  <si>
+    <t>For both rates: value equals count * 1000 / member_month_count when member_month_count is positive, and is null when it is zero. Flag a null where a value is expected, and a value where null is expected.</t>
+  </si>
+  <si>
+    <t>Tolerance 1e-6; zero-claim enrolled rows must have a rate of 0, not null.</t>
   </si>
 </sst>
 </file>
@@ -364,7 +570,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -406,30 +612,24 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
@@ -437,15 +637,13 @@
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
@@ -453,7 +651,6 @@
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -461,7 +658,6 @@
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -469,91 +665,66 @@
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -580,6 +751,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -628,19 +805,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="4" tint="0.79998"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -652,19 +829,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.79998"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -676,19 +853,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="6" tint="0.79998"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -700,19 +877,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.79998"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -724,19 +901,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="8" tint="0.79998"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -748,29 +925,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.79998"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -802,7 +988,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4" tint="0.49998"/>
       </bottom>
       <diagonal/>
     </border>
@@ -895,7 +1081,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
@@ -907,119 +1093,119 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="34" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="35" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1039,29 +1225,62 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1539,7 +1758,7 @@
     <col min="1" max="1" width="35.8083333333333" style="1" customWidth="1"/>
     <col min="2" max="2" width="23.5" style="1" customWidth="1"/>
     <col min="3" max="3" width="56.35" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.725" style="7" customWidth="1"/>
+    <col min="4" max="4" width="7.725" style="23" customWidth="1"/>
     <col min="5" max="5" width="68.6666666666667" style="1" customWidth="1"/>
     <col min="6" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
@@ -1550,38 +1769,50 @@
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="8"/>
+      <c r="D1" s="24"/>
       <c r="E1" s="2"/>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="9" t="s">
+      <c r="B2"/>
+      <c r="C2"/>
+      <c r="D2"/>
+      <c r="E2"/>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" s="9" t="s">
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="10" t="s">
         <v>3</v>
       </c>
+      <c r="B4"/>
+      <c r="C4"/>
+      <c r="D4"/>
+      <c r="E4"/>
     </row>
     <row r="6" ht="19" customHeight="1" spans="1:5">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="11" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1595,7 +1826,7 @@
       <c r="C7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="25" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="6" t="s">
@@ -1612,7 +1843,7 @@
       <c r="C8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="25" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="6" t="s">
@@ -1620,53 +1851,53 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="15" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="15" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="15" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1680,7 +1911,7 @@
       <c r="C12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="25" t="s">
         <v>12</v>
       </c>
       <c r="E12" s="6" t="s">
@@ -1697,7 +1928,7 @@
       <c r="C13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="25" t="s">
         <v>12</v>
       </c>
       <c r="E13" s="6" t="s">
@@ -1714,7 +1945,7 @@
       <c r="C14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="25" t="s">
         <v>12</v>
       </c>
       <c r="E14" s="6" t="s">
@@ -1722,36 +1953,36 @@
       </c>
     </row>
     <row r="15" ht="28.8" customHeight="1" spans="1:5">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="16" ht="28.8" customHeight="1" spans="1:5">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="15" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1765,7 +1996,7 @@
       <c r="C17" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="25" t="s">
         <v>12</v>
       </c>
       <c r="E17" s="6" t="s">
@@ -1782,7 +2013,7 @@
       <c r="C18" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="25" t="s">
         <v>12</v>
       </c>
       <c r="E18" s="6" t="s">
@@ -1790,81 +2021,81 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="15" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="15" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="15" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D22" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="15" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="24" ht="21" customHeight="1" spans="1:5">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="10"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="11"/>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="6" t="s">
@@ -1874,7 +2105,7 @@
         <v>58</v>
       </c>
       <c r="C25" s="6"/>
-      <c r="D25" s="12"/>
+      <c r="D25" s="25"/>
       <c r="E25" s="6"/>
     </row>
     <row r="26" spans="1:5">
@@ -1885,7 +2116,7 @@
         <v>60</v>
       </c>
       <c r="C26" s="6"/>
-      <c r="D26" s="12"/>
+      <c r="D26" s="25"/>
       <c r="E26" s="6"/>
     </row>
     <row r="27" spans="1:5">
@@ -1896,7 +2127,7 @@
         <v>62</v>
       </c>
       <c r="C27" s="6"/>
-      <c r="D27" s="12"/>
+      <c r="D27" s="25"/>
       <c r="E27" s="6"/>
     </row>
     <row r="28" spans="1:5">
@@ -1907,16 +2138,19 @@
         <v>64</v>
       </c>
       <c r="C28" s="6"/>
-      <c r="D28" s="12"/>
+      <c r="D28" s="25"/>
       <c r="E28" s="6"/>
     </row>
-    <row r="29" ht="28" customHeight="1" spans="1:2">
+    <row r="29" ht="28" customHeight="1" spans="1:5">
       <c r="A29" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B29" s="14" t="s">
+      <c r="B29" s="22" t="s">
         <v>66</v>
       </c>
+      <c r="C29"/>
+      <c r="D29"/>
+      <c r="E29"/>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="6" t="s">
@@ -1926,16 +2160,19 @@
         <v>68</v>
       </c>
       <c r="C30" s="6"/>
-      <c r="D30" s="12"/>
+      <c r="D30" s="25"/>
       <c r="E30" s="6"/>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:5">
       <c r="A31" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="14" t="s">
+      <c r="B31" s="22" t="s">
         <v>70</v>
       </c>
+      <c r="C31"/>
+      <c r="D31"/>
+      <c r="E31"/>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="6" t="s">
@@ -1945,7 +2182,7 @@
         <v>72</v>
       </c>
       <c r="C32" s="6"/>
-      <c r="D32" s="12"/>
+      <c r="D32" s="25"/>
       <c r="E32" s="6"/>
     </row>
     <row r="33" spans="1:5">
@@ -1956,7 +2193,7 @@
         <v>74</v>
       </c>
       <c r="C33" s="6"/>
-      <c r="D33" s="12"/>
+      <c r="D33" s="25"/>
       <c r="E33" s="6"/>
     </row>
     <row r="34" spans="1:5">
@@ -1967,7 +2204,7 @@
         <v>76</v>
       </c>
       <c r="C34" s="6"/>
-      <c r="D34" s="12"/>
+      <c r="D34" s="25"/>
       <c r="E34" s="6"/>
     </row>
     <row r="35" spans="1:5">
@@ -1978,7 +2215,7 @@
         <v>78</v>
       </c>
       <c r="C35" s="6"/>
-      <c r="D35" s="12"/>
+      <c r="D35" s="25"/>
       <c r="E35" s="6"/>
     </row>
     <row r="36" spans="1:2">
@@ -2013,10 +2250,492 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="35.8083333333333" customWidth="1"/>
+    <col min="2" max="2" width="23.5" customWidth="1"/>
+    <col min="3" max="3" width="56.35" customWidth="1"/>
+    <col min="4" max="4" width="7.725" customWidth="1"/>
+    <col min="5" max="5" width="68.6666666666667" customWidth="1"/>
+    <col min="6" max="6" width="9" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1" spans="1:5">
+      <c r="A1" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+    </row>
+    <row r="2" ht="14.4" spans="1:1">
+      <c r="A2" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" ht="14.4" spans="1:1">
+      <c r="A3" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" ht="37" customHeight="1" spans="1:1">
+      <c r="A4" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" ht="19" customHeight="1" spans="1:5">
+      <c r="A5" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1" spans="1:5">
+      <c r="A6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:5">
+      <c r="A7" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1" spans="1:5">
+      <c r="A8" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" spans="1:5">
+      <c r="A9" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1" spans="1:5">
+      <c r="A10" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" spans="1:5">
+      <c r="A11" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" spans="1:5">
+      <c r="A12" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" spans="1:5">
+      <c r="A13" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" spans="1:5">
+      <c r="A14" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" ht="28.8" spans="1:5">
+      <c r="A15" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" ht="28.8" spans="1:5">
+      <c r="A16" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" ht="28.8" spans="1:5">
+      <c r="A17" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" ht="28.8" spans="1:5">
+      <c r="A18" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" s="8" customFormat="1" ht="14.4" spans="1:5">
+      <c r="A19" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="20" s="8" customFormat="1" ht="14.4" spans="1:5">
+      <c r="A20" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" s="8" customFormat="1" ht="14.4" spans="1:5">
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="17"/>
+    </row>
+    <row r="22" ht="21" customHeight="1" spans="1:5">
+      <c r="A22" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="11"/>
+    </row>
+    <row r="23" ht="14.4" spans="1:2">
+      <c r="A23" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23" s="22" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" ht="14.4" spans="1:2">
+      <c r="A24" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="25" ht="14.4" spans="1:2">
+      <c r="A25" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="26" ht="14.4" spans="1:2">
+      <c r="A26" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="27" ht="14.4" spans="1:2">
+      <c r="A27" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" s="22" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="28" ht="14.4" spans="1:2">
+      <c r="A28" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="29" ht="14.4" spans="1:2">
+      <c r="A29" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B29" s="22" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="30" ht="14.4" spans="1:2">
+      <c r="A30" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="31" ht="14.4" spans="1:2">
+      <c r="A31" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B31" s="22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="32" ht="14.4" spans="1:2">
+      <c r="A32" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B32" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="33" ht="14.4" spans="1:2">
+      <c r="A33" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B33" s="22" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" ht="14.4" spans="1:2">
+      <c r="A34" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="35" ht="14.4" spans="1:2">
+      <c r="A35" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B35" s="22" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="36" ht="14.4" spans="1:2">
+      <c r="A36" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B36" s="22" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="37" ht="14.4" spans="1:2">
+      <c r="A37" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B37" s="22" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="38" ht="14.4" spans="1:2">
+      <c r="A38" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B38" s="22" t="s">
+        <v>131</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B38:E38"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="52.5416666666667" style="1" customWidth="1"/>
+    <col min="1" max="1" width="58.3" style="1" customWidth="1"/>
     <col min="2" max="2" width="22.0916666666667" style="1" customWidth="1"/>
     <col min="3" max="3" width="56.0833333333333" style="1" customWidth="1"/>
     <col min="4" max="4" width="15.275" style="1" customWidth="1"/>
@@ -2024,28 +2743,36 @@
     <col min="6" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:1">
+    <row r="1" ht="28" customHeight="1" spans="1:5">
       <c r="A1" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
+        <v>132</v>
+      </c>
+      <c r="B1"/>
+      <c r="C1"/>
+      <c r="D1"/>
+      <c r="E1"/>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
-        <v>84</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="B2"/>
+      <c r="C2"/>
+      <c r="D2"/>
+      <c r="E2"/>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:5">
       <c r="A4" s="4" t="s">
-        <v>85</v>
+        <v>134</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>86</v>
+        <v>135</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>87</v>
+        <v>136</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>88</v>
+        <v>137</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>8</v>
@@ -2053,87 +2780,172 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
-        <v>89</v>
+        <v>138</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>90</v>
+        <v>139</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>91</v>
+        <v>140</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>92</v>
+        <v>141</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>93</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6" ht="43.2" customHeight="1" spans="1:5">
       <c r="A6" s="6" t="s">
-        <v>94</v>
+        <v>143</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>95</v>
+        <v>144</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>96</v>
+        <v>145</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>92</v>
+        <v>141</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>97</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" ht="43.2" customHeight="1" spans="1:5">
       <c r="A7" s="5" t="s">
-        <v>98</v>
+        <v>147</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>95</v>
+        <v>144</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>99</v>
+        <v>148</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>92</v>
+        <v>141</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>100</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" ht="57.6" customHeight="1" spans="1:5">
       <c r="A8" s="6" t="s">
-        <v>101</v>
+        <v>150</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>102</v>
+        <v>151</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>103</v>
+        <v>152</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>92</v>
+        <v>141</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>104</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9" ht="43.2" customHeight="1" spans="1:5">
-      <c r="A9" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>107</v>
+      <c r="A9" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" ht="28.8" spans="1:5">
+      <c r="A10" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="11" ht="86.4" spans="1:5">
+      <c r="A11" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" ht="57.6" spans="1:5">
+      <c r="A12" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="13" ht="72" spans="1:5">
+      <c r="A13" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="14" ht="43.2" spans="1:5">
+      <c r="A14" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>